<commit_message>
Clarify starter workbook platform support
</commit_message>
<xml_diff>
--- a/Energy_Price_Comparison_Template.xlsx
+++ b/Energy_Price_Comparison_Template.xlsx
@@ -114,22 +114,34 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>No XML or manifest setup</t>
+          <t>Compatibility</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Do not use Developer tools, XML Expansion Packs, sideloading, or macros for this workbook.</t>
+          <t>Formula refresh uses WEBSERVICE and FILTERXML, which are intended for Windows desktop Excel. Use this starter on Excel for Windows, not Excel for Mac or Excel for the web.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>No XML or manifest setup</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Do not use Developer tools, XML Expansion Packs, sideloading, or macros for this workbook.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>This workbook is valid .xlsx structure, contains no embedded API key, and uses native Excel formulas.</t>
         </is>

</xml_diff>

<commit_message>
Clarify starter workbook platform support (#8)
</commit_message>
<xml_diff>
--- a/Energy_Price_Comparison_Template.xlsx
+++ b/Energy_Price_Comparison_Template.xlsx
@@ -114,22 +114,34 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>No XML or manifest setup</t>
+          <t>Compatibility</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Do not use Developer tools, XML Expansion Packs, sideloading, or macros for this workbook.</t>
+          <t>Formula refresh uses WEBSERVICE and FILTERXML, which are intended for Windows desktop Excel. Use this starter on Excel for Windows, not Excel for Mac or Excel for the web.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>No XML or manifest setup</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Do not use Developer tools, XML Expansion Packs, sideloading, or macros for this workbook.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>This workbook is valid .xlsx structure, contains no embedded API key, and uses native Excel formulas.</t>
         </is>

</xml_diff>

<commit_message>
Simplify Excel workbook fallback copy
</commit_message>
<xml_diff>
--- a/Energy_Price_Comparison_Template.xlsx
+++ b/Energy_Price_Comparison_Template.xlsx
@@ -216,7 +216,7 @@
         </is>
       </c>
       <c r="B6" s="6" t="str">
-        <f>IF($B$5="","Waiting for API key",IFERROR(IF(FILTERXML($J$2,"/oilpriceapi/status")="auth_failed","API key was not accepted. Check the key cell and try again.",FILTERXML($J$2,"/oilpriceapi/message")),"Excel blocked or did not return API data. Enable editing and external content once, then press F9."))</f>
+        <f>IF($B$5="","Waiting for API key",IFERROR(IF(FILTERXML($J$2,"/oilpriceapi/status")="auth_failed","API key was not accepted. Check the key cell and try again.",FILTERXML($J$2,"/oilpriceapi/message")),"Excel formula fetch did not return data. Use oilpriceapi.com/excel for instant download."))</f>
         <v>Waiting for API key</v>
       </c>
     </row>
@@ -327,19 +327,7 @@
       </c>
       <c r="B13" s="9" t="inlineStr">
         <is>
-          <t>Use Windows desktop Excel. Microsoft may ask to Enable Editing and Enable Content once because this downloaded workbook contacts a web endpoint.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="36" customHeight="1">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>No setup chores</t>
-        </is>
-      </c>
-      <c r="B14" s="9" t="inlineStr">
-        <is>
-          <t>No XML Expansion Packs, macros, manifest XML, Developer tools, add-in sideloading, or Trust Center catalog setup. The starter scope is WTI_USD and BRENT_CRUDE_USD.</t>
+          <t>Use the instant Excel download at oilpriceapi.com/excel if workbook formulas are blocked.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Simplify Excel workbook fallback copy (#10)
</commit_message>
<xml_diff>
--- a/Energy_Price_Comparison_Template.xlsx
+++ b/Energy_Price_Comparison_Template.xlsx
@@ -216,7 +216,7 @@
         </is>
       </c>
       <c r="B6" s="6" t="str">
-        <f>IF($B$5="","Waiting for API key",IFERROR(IF(FILTERXML($J$2,"/oilpriceapi/status")="auth_failed","API key was not accepted. Check the key cell and try again.",FILTERXML($J$2,"/oilpriceapi/message")),"Excel blocked or did not return API data. Enable editing and external content once, then press F9."))</f>
+        <f>IF($B$5="","Waiting for API key",IFERROR(IF(FILTERXML($J$2,"/oilpriceapi/status")="auth_failed","API key was not accepted. Check the key cell and try again.",FILTERXML($J$2,"/oilpriceapi/message")),"Excel formula fetch did not return data. Use oilpriceapi.com/excel for instant download."))</f>
         <v>Waiting for API key</v>
       </c>
     </row>
@@ -327,19 +327,7 @@
       </c>
       <c r="B13" s="9" t="inlineStr">
         <is>
-          <t>Use Windows desktop Excel. Microsoft may ask to Enable Editing and Enable Content once because this downloaded workbook contacts a web endpoint.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="36" customHeight="1">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>No setup chores</t>
-        </is>
-      </c>
-      <c r="B14" s="9" t="inlineStr">
-        <is>
-          <t>No XML Expansion Packs, macros, manifest XML, Developer tools, add-in sideloading, or Trust Center catalog setup. The starter scope is WTI_USD and BRENT_CRUDE_USD.</t>
+          <t>Use the instant Excel download at oilpriceapi.com/excel if workbook formulas are blocked.</t>
         </is>
       </c>
     </row>

</xml_diff>